<commit_message>
chore: remove hardcoded api secret, clean up old artifacts, fix canva flow
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,28 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/REFrameworkNET5/StudioTemplates/REFramework/contentFiles/any/any/pt2/VisualBasic/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UiPath\JobPosting_FINAL\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8C54E24-BA5C-4BF9-8DAB-2778512EC11B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01552AAD-6980-4187-B61C-8CD58C5DCAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
+    <sheet name="CanvaPoster" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="106">
   <si>
     <t>Name</t>
   </si>
@@ -160,13 +161,196 @@
   </si>
   <si>
     <t>ProcessABCQueue</t>
+  </si>
+  <si>
+    <t>InputMode</t>
+  </si>
+  <si>
+    <t>Manual</t>
+  </si>
+  <si>
+    <t>InputPath</t>
+  </si>
+  <si>
+    <t>URL hoặc Path</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>InputFilePath</t>
+  </si>
+  <si>
+    <t>Data\Input\Jobs_Local.xlsx</t>
+  </si>
+  <si>
+    <t>Path to Excel input file</t>
+  </si>
+  <si>
+    <t>InputSheetName</t>
+  </si>
+  <si>
+    <t>Sheet name containing job data</t>
+  </si>
+  <si>
+    <t>Canva_TokenFilePath</t>
+  </si>
+  <si>
+    <t>Data\Temp\canva_tokens.json</t>
+  </si>
+  <si>
+    <t>Path to saved Canva tokens (from get_canva_token.ps1)</t>
+  </si>
+  <si>
+    <t>Canva_BrandTemplateId</t>
+  </si>
+  <si>
+    <t>Canva Brand Template ID (verified)</t>
+  </si>
+  <si>
+    <t>Canva_ApiBaseUrl</t>
+  </si>
+  <si>
+    <t>https://api.canva.com/rest/v1</t>
+  </si>
+  <si>
+    <t>Canva Connect API base URL</t>
+  </si>
+  <si>
+    <t>Canva_ClientId</t>
+  </si>
+  <si>
+    <t>OC-AZ2iLEHXVW41</t>
+  </si>
+  <si>
+    <t>Canva App Client ID</t>
+  </si>
+  <si>
+    <t>Canva_ExportFormat</t>
+  </si>
+  <si>
+    <t>png</t>
+  </si>
+  <si>
+    <t>Export format: png / pdf / jpg</t>
+  </si>
+  <si>
+    <t>Canva_ExportWidth</t>
+  </si>
+  <si>
+    <t>Export width in pixels</t>
+  </si>
+  <si>
+    <t>Canva_ExportHeight</t>
+  </si>
+  <si>
+    <t>Export height in pixels</t>
+  </si>
+  <si>
+    <t>Canva_OutputFolder</t>
+  </si>
+  <si>
+    <t>Data\Output\Posters</t>
+  </si>
+  <si>
+    <t>Folder to save downloaded posters</t>
+  </si>
+  <si>
+    <t>Canva_PollIntervalMs</t>
+  </si>
+  <si>
+    <t>Milliseconds between poll requests</t>
+  </si>
+  <si>
+    <t>Canva_PollMaxAttempts</t>
+  </si>
+  <si>
+    <t>Max poll attempts before timeout</t>
+  </si>
+  <si>
+    <t>Canva_DelayBetweenJobsMs</t>
+  </si>
+  <si>
+    <t>Delay between processing each job (rate limit)</t>
+  </si>
+  <si>
+    <t>RetryCount</t>
+  </si>
+  <si>
+    <t>Number of retries on API error</t>
+  </si>
+  <si>
+    <t>CleanupTempFiles</t>
+  </si>
+  <si>
+    <t>Delete temp files after completion</t>
+  </si>
+  <si>
+    <t>GmailConnectionId</t>
+  </si>
+  <si>
+    <t>Gmail API Connection ID for sending emails with poster attached</t>
+  </si>
+  <si>
+    <t>a03a0f0a-762f-44c5-9d07-4d280413f2ed</t>
+  </si>
+  <si>
+    <t>Canva_Field_Role</t>
+  </si>
+  <si>
+    <t>Canva_Field_CareerLevel</t>
+  </si>
+  <si>
+    <t>Canva_Field_Headcount</t>
+  </si>
+  <si>
+    <t>Canva_Field_WorkLocation</t>
+  </si>
+  <si>
+    <t>Canva_Field_WorkSetup</t>
+  </si>
+  <si>
+    <t>Canva_Field_WorkSchedule</t>
+  </si>
+  <si>
+    <t>Canva_Field_Qualifications</t>
+  </si>
+  <si>
+    <t> `Drive` / `Local` / `Manual` | Chọn chế độ input |</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Career Level</t>
+  </si>
+  <si>
+    <t>Headcount</t>
+  </si>
+  <si>
+    <t>Work Location</t>
+  </si>
+  <si>
+    <t>Work Setup</t>
+  </si>
+  <si>
+    <t>Work Schedule</t>
+  </si>
+  <si>
+    <t>Qualifications</t>
+  </si>
+  <si>
+    <t>EAHHQIFhk_o</t>
+  </si>
+  <si>
+    <t>Open Demands</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -190,16 +374,41 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF13458B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -207,20 +416,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -610,15 +841,89 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="8"/>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="8"/>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="8"/>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" s="8"/>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="8"/>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" s="8"/>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A13" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="8"/>
+    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A14" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C14" s="8"/>
+    </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>
@@ -3818,4 +4123,206 @@
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C254A856-F878-4CCA-B098-E6C6D2C1CA61}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="6">
+        <v>1080</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="6">
+        <v>1080</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="6">
+        <v>3000</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="6">
+        <v>20</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="6">
+        <v>2000</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="6">
+        <v>3</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>